<commit_message>
Ajout du schéma prototype d'ensemble
</commit_message>
<xml_diff>
--- a/Hardware/Matériel.xlsx
+++ b/Hardware/Matériel.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>Nom</t>
   </si>
@@ -35,7 +35,7 @@
     <t>nombre</t>
   </si>
   <si>
-    <t>tot</t>
+    <t>somme</t>
   </si>
   <si>
     <t>ESP32</t>
@@ -59,7 +59,7 @@
     <t>Alimentation</t>
   </si>
   <si>
-    <t>TR10S05</t>
+    <t>TR10S3V3</t>
   </si>
   <si>
     <t xml:space="preserve">Écran OLED</t>
@@ -84,6 +84,45 @@
   </si>
   <si>
     <t>SLW-874744-6A-RA-N-D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diode Schottky</t>
+  </si>
+  <si>
+    <t>1N5822-T</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LED (ambre)</t>
+  </si>
+  <si>
+    <t>LTST-C150AKT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résistance 68R</t>
+  </si>
+  <si>
+    <t>AC1206JR-0768RL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résistance 120R</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> RC1206JR-07120RL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Résistance 4k7</t>
+  </si>
+  <si>
+    <t>RC1206JR-104K7L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensateur  22 uF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condensateur  47 uF</t>
+  </si>
+  <si>
+    <t>total</t>
   </si>
 </sst>
 </file>
@@ -140,7 +179,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="44" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -163,6 +202,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -714,7 +755,7 @@
         <v>1</v>
       </c>
       <c r="G4" s="7">
-        <f t="shared" ref="G4:G6" si="0">F4*E4</f>
+        <f t="shared" ref="G4:G9" si="0">F4*E4</f>
         <v>5.9400000000000004</v>
       </c>
     </row>
@@ -779,7 +820,7 @@
         <v>1</v>
       </c>
       <c r="G7" s="7">
-        <f>F7*E7</f>
+        <f t="shared" si="0"/>
         <v>5.3600000000000003</v>
       </c>
       <c r="I7" s="9"/>
@@ -801,7 +842,7 @@
         <v>2</v>
       </c>
       <c r="G8" s="7">
-        <f>F8*E8</f>
+        <f t="shared" si="0"/>
         <v>1.4199999999999999</v>
       </c>
     </row>
@@ -822,7 +863,7 @@
         <v>1</v>
       </c>
       <c r="G9" s="7">
-        <f>F9*E9</f>
+        <f t="shared" si="0"/>
         <v>5.0700000000000003</v>
       </c>
     </row>
@@ -847,8 +888,163 @@
         <v>0.40999999999999998</v>
       </c>
     </row>
+    <row r="11" ht="14.25">
+      <c r="B11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="6">
+        <v>0.87</v>
+      </c>
+      <c r="F11" s="2">
+        <v>1</v>
+      </c>
+      <c r="G11" s="7">
+        <f>F11*E11</f>
+        <v>0.87</v>
+      </c>
+    </row>
+    <row r="12" ht="14.25">
+      <c r="B12" t="s">
+        <v>24</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0.11</v>
+      </c>
+      <c r="F12" s="2">
+        <v>2</v>
+      </c>
+      <c r="G12" s="7">
+        <f>F12*E12</f>
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="13" ht="14.25">
+      <c r="B13" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E13" s="6">
+        <v>8.0000000000000002e-002</v>
+      </c>
+      <c r="F13" s="2">
+        <v>2</v>
+      </c>
+      <c r="G13" s="7">
+        <f>F13*E13</f>
+        <v>0.16</v>
+      </c>
+    </row>
     <row r="14" ht="14.25">
-      <c r="G14" s="9"/>
+      <c r="B14" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="6">
+        <v>8.0000000000000002e-002</v>
+      </c>
+      <c r="F14" s="2">
+        <v>1</v>
+      </c>
+      <c r="G14" s="7">
+        <f>F14*E14</f>
+        <v>8.0000000000000002e-002</v>
+      </c>
+    </row>
+    <row r="15" ht="14.25">
+      <c r="B15" s="10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E15" s="6">
+        <v>8.0000000000000002e-002</v>
+      </c>
+      <c r="F15" s="2">
+        <v>2</v>
+      </c>
+      <c r="G15" s="7">
+        <f>F15*E15</f>
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="16" ht="14.25">
+      <c r="B16" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="11" t="str">
+        <f>"860010272001"</f>
+        <v>860010272001</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E16" s="6">
+        <v>8.0000000000000002e-002</v>
+      </c>
+      <c r="F16" s="2">
+        <v>1</v>
+      </c>
+      <c r="G16" s="7">
+        <f>F16*E16</f>
+        <v>8.0000000000000002e-002</v>
+      </c>
+    </row>
+    <row r="17" ht="14.25">
+      <c r="B17" s="10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C17" s="11" t="str">
+        <f>"860010272003"</f>
+        <v>860010272003</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" s="6">
+        <v>8.0000000000000002e-002</v>
+      </c>
+      <c r="F17" s="2">
+        <v>1</v>
+      </c>
+      <c r="G17" s="7">
+        <f>F17*E17</f>
+        <v>8.0000000000000002e-002</v>
+      </c>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="F19" t="s">
+        <v>34</v>
+      </c>
+      <c r="G19" s="9">
+        <f>SUM(G4:G17)</f>
+        <v>31.139999999999993</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -858,10 +1054,17 @@
     <hyperlink r:id="rId4" ref="C8" tooltip=""/>
     <hyperlink r:id="rId5" ref="C9" tooltip=""/>
     <hyperlink r:id="rId6" ref="C10" tooltip=""/>
+    <hyperlink r:id="rId7" ref="C11" tooltip=""/>
+    <hyperlink r:id="rId8" ref="C12" tooltip=""/>
+    <hyperlink r:id="rId9" ref="C13" tooltip=""/>
+    <hyperlink r:id="rId10" ref="C14" tooltip=""/>
+    <hyperlink r:id="rId11" ref="C15" tooltip=""/>
+    <hyperlink r:id="rId12" ref="C16" tooltip=""/>
+    <hyperlink r:id="rId13" ref="C17" tooltip=""/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
modification liste matériel avec lien vers datasheet
</commit_message>
<xml_diff>
--- a/Hardware/Matériel.xlsx
+++ b/Hardware/Matériel.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>Nom</t>
   </si>
@@ -26,6 +26,9 @@
     <t>Ref</t>
   </si>
   <si>
+    <t>datasheet</t>
+  </si>
+  <si>
     <t>Fournisseur</t>
   </si>
   <si>
@@ -44,6 +47,9 @@
     <t>XIAO-ESP32-S3</t>
   </si>
   <si>
+    <t>./Datasheets/esp32-s3.pdf</t>
+  </si>
+  <si>
     <t>Mouser</t>
   </si>
   <si>
@@ -62,6 +68,9 @@
     <t xml:space="preserve">TSR 1-2433E</t>
   </si>
   <si>
+    <t xml:space="preserve">./Datasheets/TSR 1-2433E - tsr1e_datasheet.pdf</t>
+  </si>
+  <si>
     <t xml:space="preserve">Écran OLED</t>
   </si>
   <si>
@@ -74,36 +83,54 @@
     <t>TB0011-350-04GR</t>
   </si>
   <si>
+    <t>./Datasheets/TB0011-350-04GR.pdf</t>
+  </si>
+  <si>
     <t xml:space="preserve">transceiver UART &lt;-&gt; RS485</t>
   </si>
   <si>
     <t>MAX3485CSA+T</t>
   </si>
   <si>
+    <t>./Datasheets/MAX3483_MAX3491.pdf</t>
+  </si>
+  <si>
     <t xml:space="preserve">Switch horizontal</t>
   </si>
   <si>
     <t>SLW-874744-6A-RA-N-D</t>
   </si>
   <si>
+    <t>./Datasheets/slw_874744_6a_ra_n_d.pdf</t>
+  </si>
+  <si>
     <t xml:space="preserve">LED (ambre)</t>
   </si>
   <si>
     <t>LTST-C150AKT</t>
   </si>
   <si>
+    <t xml:space="preserve">./Datasheets/AmberLed - LTST-C150AKT.pdf</t>
+  </si>
+  <si>
     <t xml:space="preserve">Résistance 68R</t>
   </si>
   <si>
     <t>AC1206JR-0768RL</t>
   </si>
   <si>
+    <t xml:space="preserve">./Datasheets/68R - PYU_AC_51_ROHS_L.pdf</t>
+  </si>
+  <si>
     <t xml:space="preserve">Résistance 120R</t>
   </si>
   <si>
     <t xml:space="preserve"> RC1206JR-07120RL</t>
   </si>
   <si>
+    <t xml:space="preserve">./Datasheets/120R - YAGEO_PYu_RC_Group_51_RoHS_L_12.pdf</t>
+  </si>
+  <si>
     <t xml:space="preserve">Résistance 4k7</t>
   </si>
   <si>
@@ -116,16 +143,25 @@
     <t>CL31A106MBHNNNE</t>
   </si>
   <si>
+    <t xml:space="preserve">./Datasheets/Condensateur  10 uF ceram - DataSheet_CL31A106MBHNNN_20260505.pdf</t>
+  </si>
+  <si>
     <t xml:space="preserve">Condensateur  4,7 uF ceram</t>
   </si>
   <si>
-    <t>CL10A475MQ8NQWC</t>
+    <t>GRM319R61H475KA12D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">./Datasheets/Condensateur  4,7 uF ceram - Samsung_MLCC-1837944.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">Condensateur  22 uF ceram</t>
   </si>
   <si>
-    <t>GRM188R61A226ME15D</t>
+    <t>RDEC71H226MWK1H03B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">./Datasheets/Condensateur  22 uF ceram - GRM188R61A226ME15-02A.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">Condensateur  470 uF elec</t>
@@ -134,31 +170,49 @@
     <t>REF1020471M050K</t>
   </si>
   <si>
+    <t xml:space="preserve">./Datasheets/Condensateur  470 uF elec - ref-series.pdf</t>
+  </si>
+  <si>
     <t xml:space="preserve">Fusible réarmable PTC</t>
   </si>
   <si>
     <t>MF-R050</t>
   </si>
   <si>
+    <t>./Datasheets/PTC.pdf</t>
+  </si>
+  <si>
     <t xml:space="preserve">diode TVS</t>
   </si>
   <si>
+    <t xml:space="preserve">./Datasheets/diode TVS - 824500281.pdf</t>
+  </si>
+  <si>
     <t xml:space="preserve">Diode Schottky</t>
   </si>
   <si>
     <t>BX36_R1_00001</t>
   </si>
   <si>
+    <t xml:space="preserve">./Datasheets/Diode - BX36_R1_00001.pdf</t>
+  </si>
+  <si>
     <t xml:space="preserve">inductance de mode commun</t>
   </si>
   <si>
     <t>SS11VL-11050</t>
   </si>
   <si>
+    <t xml:space="preserve">./Datasheets/induct - SS11VL_11050.pdf</t>
+  </si>
+  <si>
     <t>Varistance</t>
   </si>
   <si>
     <t>MOV-20D470K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">./Datasheets/Varistance - mov20d.pdf</t>
   </si>
   <si>
     <t>total</t>
@@ -218,7 +272,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="44" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -241,7 +295,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -756,12 +809,13 @@
   <cols>
     <col customWidth="1" min="2" max="2" width="29.140625"/>
     <col bestFit="1" customWidth="1" min="3" max="3" width="27.7734375"/>
-    <col bestFit="1" customWidth="1" min="4" max="4" width="10.86328125"/>
-    <col bestFit="1" min="5" max="5" width="12.953125"/>
-    <col bestFit="1" min="6" max="6" width="9.58203125"/>
-    <col bestFit="1" min="7" max="7" width="12.953125"/>
-    <col bestFit="1" min="9" max="9" width="11.69140625"/>
-    <col bestFit="1" min="10" max="10" width="10.6328125"/>
+    <col bestFit="1" customWidth="1" min="4" max="4" width="76.75390625"/>
+    <col bestFit="1" customWidth="1" min="5" max="5" width="10.86328125"/>
+    <col bestFit="1" min="6" max="6" width="12.953125"/>
+    <col bestFit="1" min="7" max="7" width="9.58203125"/>
+    <col bestFit="1" min="8" max="8" width="12.953125"/>
+    <col bestFit="1" min="10" max="10" width="11.69140625"/>
+    <col bestFit="1" min="11" max="11" width="10.6328125"/>
   </cols>
   <sheetData>
     <row r="3" ht="14.25">
@@ -771,7 +825,7 @@
       <c r="C3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E3" s="2" t="s">
@@ -780,463 +834,540 @@
       <c r="F3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="2" t="s">
         <v>5</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="4" ht="14.25">
       <c r="B4" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="6">
+      <c r="D4" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="6">
         <v>5.9400000000000004</v>
       </c>
-      <c r="F4" s="2">
-        <v>1</v>
-      </c>
-      <c r="G4" s="7">
-        <f t="shared" ref="G4:G9" si="0">F4*E4</f>
+      <c r="G4" s="2">
+        <v>1</v>
+      </c>
+      <c r="H4" s="7">
+        <f t="shared" ref="H4:H9" si="0">G4*F4</f>
         <v>5.9400000000000004</v>
       </c>
     </row>
     <row r="5" ht="14.25">
       <c r="B5" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="6">
+        <v>12</v>
+      </c>
+      <c r="D5" s="4"/>
+      <c r="E5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="6">
         <v>8</v>
       </c>
-      <c r="F5" s="2">
-        <v>1</v>
-      </c>
-      <c r="G5" s="7">
+      <c r="G5" s="2">
+        <v>1</v>
+      </c>
+      <c r="H5" s="7">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
     </row>
     <row r="6" ht="14.25">
       <c r="B6" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="6">
+        <v>15</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="6">
         <v>2.9199999999999999</v>
       </c>
-      <c r="F6" s="2">
-        <v>1</v>
-      </c>
-      <c r="G6" s="7">
+      <c r="G6" s="2">
+        <v>1</v>
+      </c>
+      <c r="H6" s="7">
         <f t="shared" si="0"/>
         <v>2.9199999999999999</v>
       </c>
-      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
     </row>
     <row r="7" ht="14.25">
       <c r="B7" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" s="6">
+        <v>18</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="6">
         <v>5.3600000000000003</v>
       </c>
-      <c r="F7" s="2">
-        <v>1</v>
-      </c>
-      <c r="G7" s="7">
+      <c r="G7" s="2">
+        <v>1</v>
+      </c>
+      <c r="H7" s="7">
         <f t="shared" si="0"/>
         <v>5.3600000000000003</v>
       </c>
-      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
     </row>
     <row r="8" ht="14.25">
       <c r="B8" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="6">
+        <v>20</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="6">
         <v>0.70999999999999996</v>
       </c>
-      <c r="F8" s="2">
+      <c r="G8" s="2">
         <v>2</v>
       </c>
-      <c r="G8" s="7">
+      <c r="H8" s="7">
         <f t="shared" si="0"/>
         <v>1.4199999999999999</v>
       </c>
     </row>
     <row r="9" ht="14.25">
       <c r="B9" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E9" s="6">
+        <v>23</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="6">
         <v>5.0700000000000003</v>
       </c>
-      <c r="F9" s="2">
-        <v>1</v>
-      </c>
-      <c r="G9" s="7">
+      <c r="G9" s="2">
+        <v>1</v>
+      </c>
+      <c r="H9" s="7">
         <f t="shared" si="0"/>
         <v>5.0700000000000003</v>
       </c>
     </row>
     <row r="10" ht="14.25">
       <c r="B10" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="6">
+        <v>26</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="6">
         <v>0.40999999999999998</v>
       </c>
-      <c r="F10" s="2">
-        <v>1</v>
-      </c>
-      <c r="G10" s="7">
-        <f>F10*E10</f>
+      <c r="G10" s="2">
+        <v>1</v>
+      </c>
+      <c r="H10" s="7">
+        <f t="shared" ref="H10:H23" si="1">G10*F10</f>
         <v>0.40999999999999998</v>
       </c>
     </row>
     <row r="11" ht="14.25">
       <c r="B11" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" s="6">
+        <v>29</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" s="6">
         <v>0.11</v>
       </c>
-      <c r="F11" s="2">
+      <c r="G11" s="2">
         <v>2</v>
       </c>
-      <c r="G11" s="7">
-        <f>F11*E11</f>
+      <c r="H11" s="7">
+        <f t="shared" si="1"/>
         <v>0.22</v>
       </c>
     </row>
     <row r="12" ht="14.25">
       <c r="B12" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E12" s="6">
-        <v>0.080000000000000002</v>
-      </c>
-      <c r="F12" s="2">
+        <v>32</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F12" s="6">
+        <v>8.0000000000000002e-002</v>
+      </c>
+      <c r="G12" s="2">
         <v>2</v>
       </c>
-      <c r="G12" s="7">
-        <f>F12*E12</f>
+      <c r="H12" s="7">
+        <f t="shared" si="1"/>
         <v>0.16</v>
       </c>
     </row>
     <row r="13" ht="14.25">
       <c r="B13" s="10" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E13" s="6">
-        <v>0.080000000000000002</v>
-      </c>
-      <c r="F13" s="2">
-        <v>1</v>
-      </c>
-      <c r="G13" s="7">
-        <f>F13*E13</f>
-        <v>0.080000000000000002</v>
+        <v>35</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F13" s="6">
+        <v>8.0000000000000002e-002</v>
+      </c>
+      <c r="G13" s="2">
+        <v>1</v>
+      </c>
+      <c r="H13" s="7">
+        <f t="shared" si="1"/>
+        <v>8.0000000000000002e-002</v>
       </c>
     </row>
     <row r="14" ht="14.25">
       <c r="B14" s="10" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" s="6">
-        <v>0.080000000000000002</v>
-      </c>
-      <c r="F14" s="2">
+        <v>38</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="6">
+        <v>8.0000000000000002e-002</v>
+      </c>
+      <c r="G14" s="2">
         <v>2</v>
       </c>
-      <c r="G14" s="7">
-        <f>F14*E14</f>
+      <c r="H14" s="7">
+        <f t="shared" si="1"/>
         <v>0.16</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="B15" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" s="6">
+        <v>40</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="6">
         <v>0.20999999999999999</v>
       </c>
-      <c r="F15" s="2">
-        <v>1</v>
-      </c>
-      <c r="G15" s="7">
-        <f>F15*E15</f>
+      <c r="G15" s="2">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7">
+        <f t="shared" si="1"/>
         <v>0.20999999999999999</v>
       </c>
     </row>
     <row r="16" ht="14.25">
-      <c r="B16" s="11" t="s">
-        <v>32</v>
+      <c r="B16" s="10" t="s">
+        <v>42</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E16" s="6">
-        <v>0.080000000000000002</v>
-      </c>
-      <c r="F16" s="2">
-        <v>1</v>
-      </c>
-      <c r="G16" s="7">
-        <f>F16*E16</f>
-        <v>0.080000000000000002</v>
+        <v>43</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="6">
+        <v>0.17999999999999999</v>
+      </c>
+      <c r="G16" s="2">
+        <v>1</v>
+      </c>
+      <c r="H16" s="7">
+        <f t="shared" si="1"/>
+        <v>0.17999999999999999</v>
       </c>
     </row>
     <row r="17" ht="14.25">
-      <c r="B17" s="11" t="s">
-        <v>34</v>
+      <c r="B17" s="10" t="s">
+        <v>45</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E17" s="6">
-        <v>0.089999999999999997</v>
-      </c>
-      <c r="F17" s="2">
-        <v>1</v>
-      </c>
-      <c r="G17" s="7">
-        <f>F17*E17</f>
-        <v>0.089999999999999997</v>
+        <v>46</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F17" s="6">
+        <v>1.3100000000000001</v>
+      </c>
+      <c r="G17" s="2">
+        <v>1</v>
+      </c>
+      <c r="H17" s="7">
+        <f t="shared" si="1"/>
+        <v>1.3100000000000001</v>
       </c>
     </row>
     <row r="18" ht="14.25">
-      <c r="B18" s="11" t="s">
-        <v>36</v>
+      <c r="B18" s="10" t="s">
+        <v>48</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E18" s="6">
+        <v>49</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F18" s="6">
         <v>0.56999999999999995</v>
       </c>
-      <c r="F18" s="2">
-        <v>1</v>
-      </c>
-      <c r="G18" s="7">
-        <f>F18*E18</f>
+      <c r="G18" s="2">
+        <v>1</v>
+      </c>
+      <c r="H18" s="7">
+        <f t="shared" si="1"/>
         <v>0.56999999999999995</v>
       </c>
     </row>
     <row r="19" ht="14.25">
       <c r="B19" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E19" s="6">
+        <v>52</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F19" s="6">
         <v>0.32000000000000001</v>
       </c>
-      <c r="F19" s="2">
-        <v>1</v>
-      </c>
-      <c r="G19" s="7">
-        <f>F19*E19</f>
+      <c r="G19" s="2">
+        <v>1</v>
+      </c>
+      <c r="H19" s="7">
+        <f t="shared" si="1"/>
         <v>0.32000000000000001</v>
       </c>
     </row>
     <row r="20" ht="14.25">
       <c r="B20" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="12">
+        <v>54</v>
+      </c>
+      <c r="C20" s="11">
         <v>824500281</v>
       </c>
-      <c r="D20" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E20" s="6">
+      <c r="D20" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F20" s="6">
         <v>0.26000000000000001</v>
       </c>
-      <c r="F20" s="2">
-        <v>1</v>
-      </c>
-      <c r="G20" s="7">
-        <f>F20*E20</f>
+      <c r="G20" s="2">
+        <v>1</v>
+      </c>
+      <c r="H20" s="7">
+        <f t="shared" si="1"/>
         <v>0.26000000000000001</v>
       </c>
     </row>
     <row r="21" ht="14.25">
-      <c r="B21" s="13" t="s">
-        <v>41</v>
+      <c r="B21" s="12" t="s">
+        <v>56</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E21" s="6">
+        <v>57</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F21" s="6">
         <v>0.29999999999999999</v>
       </c>
-      <c r="F21" s="2">
-        <v>1</v>
-      </c>
-      <c r="G21" s="7">
-        <f>F21*E21</f>
+      <c r="G21" s="2">
+        <v>1</v>
+      </c>
+      <c r="H21" s="7">
+        <f t="shared" si="1"/>
         <v>0.29999999999999999</v>
       </c>
     </row>
     <row r="22" ht="14.25">
       <c r="B22" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E22" s="6">
+        <v>60</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F22" s="6">
         <v>1.49</v>
       </c>
-      <c r="F22" s="2">
-        <v>1</v>
-      </c>
-      <c r="G22" s="7">
-        <f>F22*E22</f>
+      <c r="G22" s="2">
+        <v>1</v>
+      </c>
+      <c r="H22" s="7">
+        <f t="shared" si="1"/>
         <v>1.49</v>
       </c>
     </row>
     <row r="23" ht="14.25">
       <c r="B23" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E23" s="6">
+        <v>63</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E23" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="F23" s="6">
         <v>0.67000000000000004</v>
       </c>
-      <c r="F23" s="2">
-        <v>1</v>
-      </c>
-      <c r="G23" s="7">
-        <f>F23*E23</f>
+      <c r="G23" s="2">
+        <v>1</v>
+      </c>
+      <c r="H23" s="7">
+        <f t="shared" si="1"/>
         <v>0.67000000000000004</v>
       </c>
     </row>
     <row r="25" ht="14.25">
-      <c r="F25" t="s">
-        <v>47</v>
-      </c>
-      <c r="G25" s="9">
-        <f>SUM(G4:G22)</f>
-        <v>33.060000000000002</v>
+      <c r="G25" t="s">
+        <v>65</v>
+      </c>
+      <c r="H25" s="9">
+        <f>SUM(H4:H22)</f>
+        <v>34.379999999999995</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C4" tooltip=""/>
-    <hyperlink r:id="rId2" ref="C6" tooltip=""/>
-    <hyperlink r:id="rId3" ref="C7" tooltip=""/>
-    <hyperlink r:id="rId4" ref="C8" tooltip=""/>
-    <hyperlink r:id="rId5" ref="C9" tooltip=""/>
-    <hyperlink r:id="rId6" ref="C10" tooltip=""/>
-    <hyperlink r:id="rId7" ref="C11" tooltip=""/>
-    <hyperlink r:id="rId8" ref="C12" tooltip=""/>
-    <hyperlink r:id="rId9" ref="C13" tooltip=""/>
-    <hyperlink r:id="rId10" ref="C14" tooltip=""/>
-    <hyperlink r:id="rId11" ref="C15" tooltip=""/>
-    <hyperlink r:id="rId12" ref="C16" tooltip=""/>
-    <hyperlink r:id="rId13" ref="C17" tooltip=""/>
-    <hyperlink r:id="rId14" ref="C18" tooltip=""/>
-    <hyperlink r:id="rId15" ref="C19" tooltip=""/>
-    <hyperlink r:id="rId16" ref="C20" tooltip=""/>
-    <hyperlink r:id="rId17" ref="C21" tooltip=""/>
-    <hyperlink r:id="rId18" ref="C22" tooltip=""/>
-    <hyperlink r:id="rId19" ref="C23" tooltip=""/>
+    <hyperlink r:id="rId2" ref="D4" tooltip=""/>
+    <hyperlink r:id="rId3" ref="C6" tooltip=""/>
+    <hyperlink r:id="rId4" ref="D6" tooltip=""/>
+    <hyperlink r:id="rId5" ref="C7" tooltip=""/>
+    <hyperlink r:id="rId6" ref="C8" tooltip=""/>
+    <hyperlink r:id="rId7" ref="D8" tooltip=""/>
+    <hyperlink r:id="rId8" ref="C9" tooltip=""/>
+    <hyperlink r:id="rId9" ref="D9" tooltip=""/>
+    <hyperlink r:id="rId10" ref="C10" tooltip=""/>
+    <hyperlink r:id="rId11" ref="D10" tooltip=""/>
+    <hyperlink r:id="rId12" ref="C11" tooltip=""/>
+    <hyperlink r:id="rId13" ref="D11" tooltip=""/>
+    <hyperlink r:id="rId14" ref="C12" tooltip=""/>
+    <hyperlink r:id="rId15" ref="D12" tooltip=""/>
+    <hyperlink r:id="rId16" ref="C13" tooltip=""/>
+    <hyperlink r:id="rId17" ref="D13" tooltip=""/>
+    <hyperlink r:id="rId18" ref="C14" tooltip=""/>
+    <hyperlink r:id="rId17" ref="D14" tooltip=""/>
+    <hyperlink r:id="rId19" ref="C15" tooltip=""/>
+    <hyperlink r:id="rId20" ref="D15" tooltip=""/>
+    <hyperlink r:id="rId21" ref="C16" tooltip=""/>
+    <hyperlink r:id="rId22" ref="D16" tooltip=""/>
+    <hyperlink r:id="rId23" ref="C17" tooltip=""/>
+    <hyperlink r:id="rId24" ref="D17" tooltip=""/>
+    <hyperlink r:id="rId25" ref="C18" tooltip=""/>
+    <hyperlink r:id="rId26" ref="D18" tooltip=""/>
+    <hyperlink r:id="rId27" ref="C19" tooltip=""/>
+    <hyperlink r:id="rId28" ref="D19" tooltip=""/>
+    <hyperlink r:id="rId29" ref="C20" tooltip=""/>
+    <hyperlink r:id="rId30" ref="D20" tooltip=""/>
+    <hyperlink r:id="rId31" ref="C21" tooltip=""/>
+    <hyperlink r:id="rId32" ref="D21" tooltip=""/>
+    <hyperlink r:id="rId33" ref="C22" tooltip=""/>
+    <hyperlink r:id="rId34" ref="D22" tooltip=""/>
+    <hyperlink r:id="rId35" ref="C23" tooltip=""/>
+    <hyperlink r:id="rId36" ref="D23" tooltip=""/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>

<commit_message>
Ajout de footprint + STEP files
</commit_message>
<xml_diff>
--- a/Hardware/Matériel.xlsx
+++ b/Hardware/Matériel.xlsx
@@ -9,6 +9,7 @@
     <sheet name="Liste de matériels (prototype)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Commandes" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="BOM" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="XIAO ESP32" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr/>
   <extLst>
@@ -18,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="145">
   <si>
     <t>Nom</t>
   </si>
@@ -74,7 +75,7 @@
     <t xml:space="preserve">Écran OLED</t>
   </si>
   <si>
-    <t xml:space="preserve">DST-015 (OLED based SSD1305)</t>
+    <t xml:space="preserve">DST-015 (OLED SSD1305)</t>
   </si>
   <si>
     <t>Bornier</t>
@@ -143,7 +144,7 @@
     <t>CL31A106MBHNNNE</t>
   </si>
   <si>
-    <t xml:space="preserve">./Datasheets/Condensateur  10 uF ceram - DataSheet_CL31A106MBHNNN_20260505.pdf</t>
+    <t>./Datasheets/DataSheet_CL31A106MBHNNN_20260505.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">Condensateur  4,7 uF ceram</t>
@@ -215,7 +216,244 @@
     <t xml:space="preserve">./Datasheets/Varistance - mov20d.pdf</t>
   </si>
   <si>
+    <t xml:space="preserve">inductance torique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">./Datasheets/induct - 7447060.pdf</t>
+  </si>
+  <si>
     <t>total</t>
+  </si>
+  <si>
+    <t>TOUCH1</t>
+  </si>
+  <si>
+    <t>A0</t>
+  </si>
+  <si>
+    <t>GPIO1</t>
+  </si>
+  <si>
+    <t>D0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XIAO ESP32-S3</t>
+  </si>
+  <si>
+    <t>5V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dual-core 240MHz</t>
+  </si>
+  <si>
+    <t>TOUCH2</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>GPIO2</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8MB PSRAM</t>
+  </si>
+  <si>
+    <t>TOUCH3</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>GPIO3</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>3V3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8MB Flash</t>
+  </si>
+  <si>
+    <t>TOUCH4</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>GPIO4</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>D10</t>
+  </si>
+  <si>
+    <t>GPIO9</t>
+  </si>
+  <si>
+    <t>A10</t>
+  </si>
+  <si>
+    <t>MOSI</t>
+  </si>
+  <si>
+    <t>TOUCH9</t>
+  </si>
+  <si>
+    <t>https://wiki.seeedstudio.com/xiao_esp32s3_getting_started/</t>
+  </si>
+  <si>
+    <t>TOUCH5</t>
+  </si>
+  <si>
+    <t>SDA</t>
+  </si>
+  <si>
+    <t>A4</t>
+  </si>
+  <si>
+    <t>GPIO5</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
+  <si>
+    <t>D9</t>
+  </si>
+  <si>
+    <t>GPIO8</t>
+  </si>
+  <si>
+    <t>A9</t>
+  </si>
+  <si>
+    <t>MISO</t>
+  </si>
+  <si>
+    <t>TOUCH8</t>
+  </si>
+  <si>
+    <t>TOUCH6</t>
+  </si>
+  <si>
+    <t>SCL</t>
+  </si>
+  <si>
+    <t>A5</t>
+  </si>
+  <si>
+    <t>GPIO6</t>
+  </si>
+  <si>
+    <t>D5</t>
+  </si>
+  <si>
+    <t>D8</t>
+  </si>
+  <si>
+    <t>GPIO7</t>
+  </si>
+  <si>
+    <t>A8</t>
+  </si>
+  <si>
+    <t>SCK</t>
+  </si>
+  <si>
+    <t>TOUCH7</t>
+  </si>
+  <si>
+    <t>TX</t>
+  </si>
+  <si>
+    <t>GPIO43</t>
+  </si>
+  <si>
+    <t>D6</t>
+  </si>
+  <si>
+    <t>D7</t>
+  </si>
+  <si>
+    <t>GPIO44</t>
+  </si>
+  <si>
+    <t>RX</t>
+  </si>
+  <si>
+    <t>LP_GPIO1</t>
+  </si>
+  <si>
+    <t>GPIO0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">XIAO ESP32-C6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dual-core 160MHz</t>
+  </si>
+  <si>
+    <t>LP_GPIO2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">512KB SRAM</t>
+  </si>
+  <si>
+    <t>SDIO_DATA1</t>
+  </si>
+  <si>
+    <t>GPIO21</t>
+  </si>
+  <si>
+    <t>GPIO18</t>
+  </si>
+  <si>
+    <t>SDIO_CMD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 MB Flash</t>
+  </si>
+  <si>
+    <t>SDIO_DATA2</t>
+  </si>
+  <si>
+    <t>GPIO22</t>
+  </si>
+  <si>
+    <t>GPIO20</t>
+  </si>
+  <si>
+    <t>SDIO_DATA0</t>
+  </si>
+  <si>
+    <t>https://wiki.seeedstudio.com/xiao_esp32C6_getting_started/</t>
+  </si>
+  <si>
+    <t>SDIO_DATA3</t>
+  </si>
+  <si>
+    <t>GPIO23</t>
+  </si>
+  <si>
+    <t>GPIO19</t>
+  </si>
+  <si>
+    <t>SDIO_CLK</t>
+  </si>
+  <si>
+    <t>GPIO16</t>
+  </si>
+  <si>
+    <t>GPIO17</t>
   </si>
 </sst>
 </file>
@@ -225,10 +463,31 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$CHF-100C]_-;\-* #,##0.00\ [$CHF-100C]_-;_-* &quot;-&quot;??\ [$CHF-100C]_-;_-@_-"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.000000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10.000000"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10.000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10.000000"/>
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
@@ -237,15 +496,6 @@
       <sz val="11.000000"/>
       <color theme="10"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11.000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="11.000000"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -272,35 +522,65 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="44" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="25">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="164" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="164" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
+    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1">
+      <protection hidden="0" locked="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="1" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" textRotation="180" vertical="center"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" textRotation="180" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="1" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="1" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
-      <protection hidden="0" locked="1"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" textRotation="180" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" textRotation="180" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -318,6 +598,116 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:w="http://schemas.openxmlformats.org/wordprocessingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>563942</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>78581</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="3962752" cy="1844035"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="498148791" name=""/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip r:embed="rId1"/>
+        <a:srcRect l="0" t="9115" r="0" b="37357"/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm flipH="0" flipV="0">
+          <a:off x="6107492" y="983455"/>
+          <a:ext cx="3962752" cy="1844035"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>473659</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>162251</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>8905</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>181575</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="0" name=""/>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr bwMode="auto">
+        <a:xfrm flipH="0" flipV="0">
+          <a:off x="6017209" y="2876876"/>
+          <a:ext cx="4412045" cy="1647498"/>
+          <a:chOff x="0" y="0"/>
+          <a:chExt cx="4412045" cy="1654693"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="630608922" name=""/>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill rotWithShape="1">
+          <a:blip r:embed="rId2"/>
+          <a:srcRect l="0" t="0" r="0" b="55890"/>
+          <a:stretch/>
+        </xdr:blipFill>
+        <xdr:spPr bwMode="auto">
+          <a:xfrm flipH="0" flipV="0">
+            <a:off x="0" y="0"/>
+            <a:ext cx="4412045" cy="1582228"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="632672839" name=""/>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill rotWithShape="1">
+          <a:blip r:embed="rId3"/>
+          <a:srcRect l="0" t="95959" r="0" b="0"/>
+          <a:stretch/>
+        </xdr:blipFill>
+        <xdr:spPr bwMode="auto">
+          <a:xfrm flipH="0" flipV="0">
+            <a:off x="0" y="1509763"/>
+            <a:ext cx="4412045" cy="144929"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme.xml><?xml version="1.0" encoding="utf-8"?>
@@ -803,17 +1193,17 @@
   <sheetPr>
     <tabColor theme="4" tint="0"/>
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
   </sheetPr>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="29.140625"/>
-    <col bestFit="1" customWidth="1" min="3" max="3" width="27.7734375"/>
-    <col bestFit="1" customWidth="1" min="4" max="4" width="76.75390625"/>
-    <col bestFit="1" customWidth="1" min="5" max="5" width="10.86328125"/>
-    <col bestFit="1" min="6" max="6" width="12.953125"/>
-    <col bestFit="1" min="7" max="7" width="9.58203125"/>
-    <col bestFit="1" min="8" max="8" width="12.953125"/>
+    <col bestFit="1" customWidth="1" min="2" max="2" width="24.29296875"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" width="20.03125"/>
+    <col bestFit="1" customWidth="1" min="4" max="4" width="59.4140625"/>
+    <col bestFit="1" customWidth="1" min="5" max="5" width="9.75390625"/>
+    <col bestFit="1" customWidth="1" min="6" max="6" width="11.62109375"/>
+    <col bestFit="1" min="7" max="7" width="6.94140625"/>
+    <col bestFit="1" customWidth="1" min="8" max="8" width="11.62109375"/>
     <col bestFit="1" min="10" max="10" width="11.69140625"/>
     <col bestFit="1" min="11" max="11" width="10.6328125"/>
   </cols>
@@ -842,408 +1232,408 @@
       </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="B4" t="s">
+      <c r="B4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F4" s="6">
+      <c r="F4" s="7">
         <v>5.9400000000000004</v>
       </c>
       <c r="G4" s="2">
         <v>1</v>
       </c>
-      <c r="H4" s="7">
+      <c r="H4" s="8">
         <f t="shared" ref="H4:H9" si="0">G4*F4</f>
         <v>5.9400000000000004</v>
       </c>
     </row>
     <row r="5" ht="14.25">
-      <c r="B5" t="s">
+      <c r="B5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D5" s="4"/>
-      <c r="E5" s="8" t="s">
+      <c r="D5" s="5"/>
+      <c r="E5" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="7">
         <v>8</v>
       </c>
       <c r="G5" s="2">
         <v>1</v>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="8">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="K5" s="9"/>
+      <c r="K5" s="10"/>
     </row>
     <row r="6" ht="14.25">
-      <c r="B6" t="s">
+      <c r="B6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="6">
+      <c r="F6" s="7">
         <v>2.9199999999999999</v>
       </c>
       <c r="G6" s="2">
         <v>1</v>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="8">
         <f t="shared" si="0"/>
         <v>2.9199999999999999</v>
       </c>
-      <c r="J6" s="9"/>
+      <c r="J6" s="10"/>
     </row>
     <row r="7" ht="14.25">
-      <c r="B7" t="s">
+      <c r="B7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="5" t="s">
+      <c r="D7" s="5"/>
+      <c r="E7" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F7" s="6">
+      <c r="F7" s="7">
         <v>5.3600000000000003</v>
       </c>
       <c r="G7" s="2">
         <v>1</v>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="8">
         <f t="shared" si="0"/>
         <v>5.3600000000000003</v>
       </c>
-      <c r="J7" s="9"/>
+      <c r="J7" s="10"/>
     </row>
     <row r="8" ht="14.25">
-      <c r="B8" t="s">
+      <c r="B8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="4" t="s">
+      <c r="C8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="D8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="6">
+      <c r="F8" s="7">
         <v>0.70999999999999996</v>
       </c>
       <c r="G8" s="2">
         <v>2</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="8">
         <f t="shared" si="0"/>
         <v>1.4199999999999999</v>
       </c>
     </row>
     <row r="9" ht="14.25">
-      <c r="B9" t="s">
+      <c r="B9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="6">
+      <c r="F9" s="7">
         <v>5.0700000000000003</v>
       </c>
       <c r="G9" s="2">
         <v>1</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="8">
         <f t="shared" si="0"/>
         <v>5.0700000000000003</v>
       </c>
     </row>
     <row r="10" ht="14.25">
-      <c r="B10" t="s">
+      <c r="B10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="D10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F10" s="6">
+      <c r="F10" s="7">
         <v>0.40999999999999998</v>
       </c>
       <c r="G10" s="2">
         <v>1</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="8">
         <f t="shared" ref="H10:H23" si="1">G10*F10</f>
         <v>0.40999999999999998</v>
       </c>
     </row>
     <row r="11" ht="14.25">
-      <c r="B11" t="s">
+      <c r="B11" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F11" s="6">
+      <c r="F11" s="7">
         <v>0.11</v>
       </c>
       <c r="G11" s="2">
         <v>2</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="8">
         <f t="shared" si="1"/>
         <v>0.22</v>
       </c>
     </row>
     <row r="12" ht="14.25">
-      <c r="B12" t="s">
+      <c r="B12" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="4" t="s">
+      <c r="D12" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F12" s="6">
+      <c r="F12" s="7">
         <v>8.0000000000000002e-002</v>
       </c>
       <c r="G12" s="2">
         <v>2</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="8">
         <f t="shared" si="1"/>
         <v>0.16</v>
       </c>
     </row>
     <row r="13" ht="14.25">
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="6">
+      <c r="F13" s="7">
         <v>8.0000000000000002e-002</v>
       </c>
       <c r="G13" s="2">
         <v>1</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="8">
         <f t="shared" si="1"/>
         <v>8.0000000000000002e-002</v>
       </c>
     </row>
     <row r="14" ht="14.25">
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="C14" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="4" t="s">
+      <c r="D14" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F14" s="6">
+      <c r="F14" s="7">
         <v>8.0000000000000002e-002</v>
       </c>
       <c r="G14" s="2">
         <v>2</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="8">
         <f t="shared" si="1"/>
         <v>0.16</v>
       </c>
     </row>
     <row r="15" ht="14.25">
-      <c r="B15" t="s">
+      <c r="B15" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="C15" s="4" t="s">
+      <c r="C15" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="4" t="s">
+      <c r="D15" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F15" s="6">
+      <c r="F15" s="7">
         <v>0.20999999999999999</v>
       </c>
       <c r="G15" s="2">
         <v>1</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="8">
         <f t="shared" si="1"/>
         <v>0.20999999999999999</v>
       </c>
     </row>
     <row r="16" ht="14.25">
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F16" s="6">
+      <c r="F16" s="7">
         <v>0.17999999999999999</v>
       </c>
       <c r="G16" s="2">
         <v>1</v>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="8">
         <f t="shared" si="1"/>
         <v>0.17999999999999999</v>
       </c>
     </row>
     <row r="17" ht="14.25">
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C17" s="4" t="s">
+      <c r="C17" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="D17" s="4" t="s">
+      <c r="D17" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="E17" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F17" s="6">
+      <c r="F17" s="7">
         <v>1.3100000000000001</v>
       </c>
       <c r="G17" s="2">
         <v>1</v>
       </c>
-      <c r="H17" s="7">
+      <c r="H17" s="8">
         <f t="shared" si="1"/>
         <v>1.3100000000000001</v>
       </c>
     </row>
     <row r="18" ht="14.25">
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E18" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F18" s="6">
+      <c r="F18" s="7">
         <v>0.56999999999999995</v>
       </c>
       <c r="G18" s="2">
         <v>1</v>
       </c>
-      <c r="H18" s="7">
+      <c r="H18" s="8">
         <f t="shared" si="1"/>
         <v>0.56999999999999995</v>
       </c>
     </row>
     <row r="19" ht="14.25">
-      <c r="B19" t="s">
+      <c r="B19" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C19" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="D19" s="4" t="s">
+      <c r="D19" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F19" s="6">
+      <c r="F19" s="7">
         <v>0.32000000000000001</v>
       </c>
       <c r="G19" s="2">
         <v>1</v>
       </c>
-      <c r="H19" s="7">
+      <c r="H19" s="8">
         <f t="shared" si="1"/>
         <v>0.32000000000000001</v>
       </c>
     </row>
     <row r="20" ht="14.25">
-      <c r="B20" t="s">
+      <c r="B20" s="4" t="s">
         <v>54</v>
       </c>
       <c r="C20" s="11">
         <v>824500281</v>
       </c>
-      <c r="D20" s="4" t="s">
+      <c r="D20" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="E20" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F20" s="6">
+      <c r="F20" s="7">
         <v>0.26000000000000001</v>
       </c>
       <c r="G20" s="2">
         <v>1</v>
       </c>
-      <c r="H20" s="7">
+      <c r="H20" s="8">
         <f t="shared" si="1"/>
         <v>0.26000000000000001</v>
       </c>
@@ -1252,81 +1642,112 @@
       <c r="B21" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="C21" s="4" t="s">
+      <c r="C21" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="D21" s="4" t="s">
+      <c r="D21" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="E21" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F21" s="6">
+      <c r="F21" s="7">
         <v>0.29999999999999999</v>
       </c>
       <c r="G21" s="2">
         <v>1</v>
       </c>
-      <c r="H21" s="7">
+      <c r="H21" s="8">
         <f t="shared" si="1"/>
         <v>0.29999999999999999</v>
       </c>
     </row>
     <row r="22" ht="14.25">
-      <c r="B22" t="s">
+      <c r="B22" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="C22" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D22" s="4" t="s">
+      <c r="D22" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="E22" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F22" s="6">
+      <c r="F22" s="7">
         <v>1.49</v>
       </c>
       <c r="G22" s="2">
         <v>1</v>
       </c>
-      <c r="H22" s="7">
+      <c r="H22" s="8">
         <f t="shared" si="1"/>
         <v>1.49</v>
       </c>
     </row>
     <row r="23" ht="14.25">
-      <c r="B23" t="s">
+      <c r="B23" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="C23" s="4" t="s">
+      <c r="C23" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="D23" s="4" t="s">
+      <c r="D23" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="E23" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F23" s="6">
+      <c r="F23" s="7">
         <v>0.67000000000000004</v>
       </c>
       <c r="G23" s="2">
         <v>1</v>
       </c>
-      <c r="H23" s="7">
+      <c r="H23" s="8">
         <f t="shared" si="1"/>
         <v>0.67000000000000004</v>
       </c>
     </row>
+    <row r="24" ht="14.25">
+      <c r="B24" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C24" s="14">
+        <v>7447060</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="F24" s="7">
+        <v>2.0600000000000001</v>
+      </c>
+      <c r="G24" s="2">
+        <v>1</v>
+      </c>
+      <c r="H24" s="8">
+        <f>G24*F24</f>
+        <v>2.0600000000000001</v>
+      </c>
+    </row>
     <row r="25" ht="14.25">
-      <c r="G25" t="s">
-        <v>65</v>
-      </c>
-      <c r="H25" s="9">
-        <f>SUM(H4:H22)</f>
-        <v>34.379999999999995</v>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+    </row>
+    <row r="27" ht="14.25">
+      <c r="G27" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="H27" s="16">
+        <f>SUM(H4:H24)</f>
+        <v>37.109999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -1368,10 +1789,12 @@
     <hyperlink r:id="rId34" ref="D22" tooltip=""/>
     <hyperlink r:id="rId35" ref="C23" tooltip=""/>
     <hyperlink r:id="rId36" ref="D23" tooltip=""/>
+    <hyperlink r:id="rId37" ref="C24" tooltip=""/>
+    <hyperlink r:id="rId38" ref="D24" tooltip=""/>
   </hyperlinks>
   <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <pageMargins left="0.25196850393700787" right="0.25196850393700787" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="98" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
 </file>
@@ -1383,7 +1806,7 @@
     <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
     <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
   </sheetPr>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData/>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
@@ -1406,4 +1829,398 @@
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+  <sheetPr>
+    <tabColor indexed="2"/>
+    <outlinePr applyStyles="0" summaryBelow="1" summaryRight="1" showOutlineSymbols="1"/>
+    <pageSetUpPr autoPageBreaks="1" fitToPage="0"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col bestFit="1" min="2" max="2" width="11.7421875"/>
+    <col bestFit="1" min="3" max="3" width="9.18359375"/>
+    <col bestFit="1" min="4" max="4" width="4.140625"/>
+    <col bestFit="1" min="5" max="5" width="7.23046875"/>
+    <col bestFit="1" min="6" max="6" width="3.0625"/>
+    <col bestFit="1" min="8" max="8" width="4.68359375"/>
+    <col bestFit="1" min="9" max="9" width="7.23046875"/>
+    <col bestFit="1" min="10" max="10" width="4.07421875"/>
+    <col bestFit="1" min="11" max="11" width="5.421875"/>
+    <col bestFit="1" min="12" max="12" width="7.97265625"/>
+  </cols>
+  <sheetData>
+    <row r="8" ht="14.25">
+      <c r="C8" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="F8" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="G8" s="19" t="s">
+        <v>72</v>
+      </c>
+      <c r="H8" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="U8" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" ht="14.25">
+      <c r="C9" s="17" t="s">
+        <v>75</v>
+      </c>
+      <c r="D9" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="17" t="s">
+        <v>77</v>
+      </c>
+      <c r="F9" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="G9" s="21"/>
+      <c r="H9" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="U9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" ht="14.25">
+      <c r="C10" s="17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>82</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="F10" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="G10" s="21"/>
+      <c r="H10" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="U10" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" ht="14.25">
+      <c r="C11" s="17" t="s">
+        <v>87</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>88</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>90</v>
+      </c>
+      <c r="G11" s="21"/>
+      <c r="H11" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="I11" t="s">
+        <v>92</v>
+      </c>
+      <c r="J11" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="K11" t="s">
+        <v>94</v>
+      </c>
+      <c r="L11" t="s">
+        <v>95</v>
+      </c>
+      <c r="U11" s="15" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" ht="14.25">
+      <c r="B12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C12" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="D12" s="17" t="s">
+        <v>99</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>100</v>
+      </c>
+      <c r="F12" s="17" t="s">
+        <v>101</v>
+      </c>
+      <c r="G12" s="21"/>
+      <c r="H12" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="I12" t="s">
+        <v>103</v>
+      </c>
+      <c r="J12" t="s">
+        <v>104</v>
+      </c>
+      <c r="K12" t="s">
+        <v>105</v>
+      </c>
+      <c r="L12" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="13" ht="14.25">
+      <c r="B13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C13" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>109</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>110</v>
+      </c>
+      <c r="F13" s="17" t="s">
+        <v>111</v>
+      </c>
+      <c r="G13" s="21"/>
+      <c r="H13" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="I13" t="s">
+        <v>113</v>
+      </c>
+      <c r="J13" t="s">
+        <v>114</v>
+      </c>
+      <c r="K13" t="s">
+        <v>115</v>
+      </c>
+      <c r="L13" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="14" ht="14.25">
+      <c r="C14" s="18"/>
+      <c r="D14" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="E14" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="F14" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="G14" s="21"/>
+      <c r="H14" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="I14" t="s">
+        <v>121</v>
+      </c>
+      <c r="J14" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="17" ht="14.25">
+      <c r="O17" s="20"/>
+    </row>
+    <row r="18" ht="14.25">
+      <c r="B18" t="s">
+        <v>123</v>
+      </c>
+      <c r="D18" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="E18" t="s">
+        <v>124</v>
+      </c>
+      <c r="F18" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="G18" s="23" t="s">
+        <v>125</v>
+      </c>
+      <c r="H18" s="20" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="19" ht="14.25">
+      <c r="B19" t="s">
+        <v>123</v>
+      </c>
+      <c r="D19" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="F19" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="G19" s="24"/>
+      <c r="H19" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="U19" s="13" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="20" ht="14.25">
+      <c r="B20" t="s">
+        <v>127</v>
+      </c>
+      <c r="D20" s="18" t="s">
+        <v>82</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="F20" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="G20" s="24"/>
+      <c r="H20" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="U20" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="21" ht="14.25">
+      <c r="B21" t="s">
+        <v>129</v>
+      </c>
+      <c r="E21" t="s">
+        <v>130</v>
+      </c>
+      <c r="F21" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="G21" s="24"/>
+      <c r="H21" s="20" t="s">
+        <v>91</v>
+      </c>
+      <c r="I21" t="s">
+        <v>131</v>
+      </c>
+      <c r="K21" t="s">
+        <v>94</v>
+      </c>
+      <c r="L21" t="s">
+        <v>132</v>
+      </c>
+      <c r="U21" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="22" ht="14.25">
+      <c r="B22" t="s">
+        <v>134</v>
+      </c>
+      <c r="C22" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="E22" t="s">
+        <v>135</v>
+      </c>
+      <c r="F22" s="18" t="s">
+        <v>101</v>
+      </c>
+      <c r="G22" s="24"/>
+      <c r="H22" s="20" t="s">
+        <v>102</v>
+      </c>
+      <c r="I22" t="s">
+        <v>136</v>
+      </c>
+      <c r="K22" t="s">
+        <v>105</v>
+      </c>
+      <c r="L22" t="s">
+        <v>137</v>
+      </c>
+      <c r="U22" s="15" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="23" ht="14.25">
+      <c r="B23" t="s">
+        <v>139</v>
+      </c>
+      <c r="C23" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="F23" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="G23" s="24"/>
+      <c r="H23" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="I23" t="s">
+        <v>141</v>
+      </c>
+      <c r="K23" t="s">
+        <v>115</v>
+      </c>
+      <c r="L23" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="24" ht="14.25">
+      <c r="D24" t="s">
+        <v>117</v>
+      </c>
+      <c r="E24" t="s">
+        <v>143</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>119</v>
+      </c>
+      <c r="G24" s="24"/>
+      <c r="H24" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="I24" t="s">
+        <v>144</v>
+      </c>
+      <c r="J24" t="s">
+        <v>122</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="G8:G14"/>
+    <mergeCell ref="G18:G24"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink r:id="rId1" ref="U11"/>
+    <hyperlink r:id="rId2" ref="U22"/>
+  </hyperlinks>
+  <printOptions headings="0" gridLines="0"/>
+  <pageMargins left="0.70078740157480324" right="0.70078740157480324" top="0.75196850393700787" bottom="0.75196850393700787" header="0.29999999999999999" footer="0.29999999999999999"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
+  <headerFooter/>
+  <drawing r:id="rId3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Mise a jour de la documentation technique
</commit_message>
<xml_diff>
--- a/Hardware/Matériel.xlsx
+++ b/Hardware/Matériel.xlsx
@@ -522,7 +522,7 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf fontId="0" fillId="2" borderId="0" numFmtId="44" applyNumberFormat="1" applyFont="0" applyFill="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="20">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -562,25 +562,10 @@
       <alignment horizontal="right"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" textRotation="180" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" textRotation="180" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" textRotation="180" vertical="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" textRotation="180" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -607,7 +592,7 @@
       <xdr:col>12</xdr:col>
       <xdr:colOff>563942</xdr:colOff>
       <xdr:row>5</xdr:row>
-      <xdr:rowOff>78581</xdr:rowOff>
+      <xdr:rowOff>78580</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="3962752" cy="1844035"/>
     <xdr:pic>
@@ -645,7 +630,7 @@
       <xdr:col>20</xdr:col>
       <xdr:colOff>8905</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>181575</xdr:rowOff>
+      <xdr:rowOff>181574</xdr:rowOff>
     </xdr:to>
     <xdr:grpSp>
       <xdr:nvGrpSpPr>
@@ -1394,7 +1379,7 @@
         <v>1</v>
       </c>
       <c r="H10" s="8">
-        <f t="shared" ref="H10:H23" si="1">G10*F10</f>
+        <f t="shared" ref="H10:H24" si="1">G10*F10</f>
         <v>0.40999999999999998</v>
       </c>
     </row>
@@ -1730,7 +1715,7 @@
         <v>1</v>
       </c>
       <c r="H24" s="8">
-        <f>G24*F24</f>
+        <f t="shared" si="1"/>
         <v>2.0600000000000001</v>
       </c>
     </row>
@@ -1856,19 +1841,19 @@
       <c r="C8" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="17" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" s="17" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="F8" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="G8" s="19" t="s">
+      <c r="G8" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="H8" s="20" t="s">
+      <c r="H8" s="19" t="s">
         <v>73</v>
       </c>
       <c r="U8" t="s">
@@ -1885,11 +1870,11 @@
       <c r="E9" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="F9" s="18" t="s">
+      <c r="F9" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="G9" s="21"/>
-      <c r="H9" s="20" t="s">
+      <c r="G9" s="18"/>
+      <c r="H9" s="19" t="s">
         <v>79</v>
       </c>
       <c r="U9" t="s">
@@ -1909,8 +1894,8 @@
       <c r="F10" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="G10" s="21"/>
-      <c r="H10" s="20" t="s">
+      <c r="G10" s="18"/>
+      <c r="H10" s="19" t="s">
         <v>85</v>
       </c>
       <c r="U10" t="s">
@@ -1930,14 +1915,14 @@
       <c r="F11" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="G11" s="21"/>
-      <c r="H11" s="20" t="s">
+      <c r="G11" s="18"/>
+      <c r="H11" s="19" t="s">
         <v>91</v>
       </c>
       <c r="I11" t="s">
         <v>92</v>
       </c>
-      <c r="J11" s="22" t="s">
+      <c r="J11" s="19" t="s">
         <v>93</v>
       </c>
       <c r="K11" t="s">
@@ -1954,7 +1939,7 @@
       <c r="B12" t="s">
         <v>97</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="17" t="s">
         <v>98</v>
       </c>
       <c r="D12" s="17" t="s">
@@ -1966,8 +1951,8 @@
       <c r="F12" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="G12" s="21"/>
-      <c r="H12" s="20" t="s">
+      <c r="G12" s="18"/>
+      <c r="H12" s="19" t="s">
         <v>102</v>
       </c>
       <c r="I12" t="s">
@@ -1987,7 +1972,7 @@
       <c r="B13" t="s">
         <v>107</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="17" t="s">
         <v>108</v>
       </c>
       <c r="D13" s="17" t="s">
@@ -1999,8 +1984,8 @@
       <c r="F13" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="G13" s="21"/>
-      <c r="H13" s="20" t="s">
+      <c r="G13" s="18"/>
+      <c r="H13" s="19" t="s">
         <v>112</v>
       </c>
       <c r="I13" t="s">
@@ -2017,18 +2002,18 @@
       </c>
     </row>
     <row r="14" ht="14.25">
-      <c r="C14" s="18"/>
-      <c r="D14" s="18" t="s">
+      <c r="C14" s="17"/>
+      <c r="D14" s="17" t="s">
         <v>117</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="E14" s="17" t="s">
         <v>118</v>
       </c>
       <c r="F14" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="G14" s="21"/>
-      <c r="H14" s="20" t="s">
+      <c r="G14" s="18"/>
+      <c r="H14" s="19" t="s">
         <v>120</v>
       </c>
       <c r="I14" t="s">
@@ -2039,25 +2024,25 @@
       </c>
     </row>
     <row r="17" ht="14.25">
-      <c r="O17" s="20"/>
+      <c r="O17" s="19"/>
     </row>
     <row r="18" ht="14.25">
       <c r="B18" t="s">
         <v>123</v>
       </c>
-      <c r="D18" s="18" t="s">
+      <c r="D18" s="17" t="s">
         <v>69</v>
       </c>
       <c r="E18" t="s">
         <v>124</v>
       </c>
-      <c r="F18" s="18" t="s">
+      <c r="F18" s="17" t="s">
         <v>71</v>
       </c>
-      <c r="G18" s="23" t="s">
+      <c r="G18" s="18" t="s">
         <v>125</v>
       </c>
-      <c r="H18" s="20" t="s">
+      <c r="H18" s="19" t="s">
         <v>73</v>
       </c>
     </row>
@@ -2065,17 +2050,17 @@
       <c r="B19" t="s">
         <v>123</v>
       </c>
-      <c r="D19" s="18" t="s">
+      <c r="D19" s="17" t="s">
         <v>76</v>
       </c>
       <c r="E19" s="13" t="s">
         <v>70</v>
       </c>
-      <c r="F19" s="18" t="s">
+      <c r="F19" s="17" t="s">
         <v>78</v>
       </c>
-      <c r="G19" s="24"/>
-      <c r="H19" s="20" t="s">
+      <c r="G19" s="18"/>
+      <c r="H19" s="19" t="s">
         <v>79</v>
       </c>
       <c r="U19" s="13" t="s">
@@ -2086,17 +2071,17 @@
       <c r="B20" t="s">
         <v>127</v>
       </c>
-      <c r="D20" s="18" t="s">
+      <c r="D20" s="17" t="s">
         <v>82</v>
       </c>
       <c r="E20" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="F20" s="18" t="s">
+      <c r="F20" s="17" t="s">
         <v>84</v>
       </c>
-      <c r="G20" s="24"/>
-      <c r="H20" s="20" t="s">
+      <c r="G20" s="18"/>
+      <c r="H20" s="19" t="s">
         <v>85</v>
       </c>
       <c r="U20" t="s">
@@ -2110,11 +2095,11 @@
       <c r="E21" t="s">
         <v>130</v>
       </c>
-      <c r="F21" s="18" t="s">
+      <c r="F21" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="G21" s="24"/>
-      <c r="H21" s="20" t="s">
+      <c r="G21" s="18"/>
+      <c r="H21" s="19" t="s">
         <v>91</v>
       </c>
       <c r="I21" t="s">
@@ -2134,17 +2119,17 @@
       <c r="B22" t="s">
         <v>134</v>
       </c>
-      <c r="C22" s="18" t="s">
+      <c r="C22" s="17" t="s">
         <v>98</v>
       </c>
       <c r="E22" t="s">
         <v>135</v>
       </c>
-      <c r="F22" s="18" t="s">
+      <c r="F22" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="G22" s="24"/>
-      <c r="H22" s="20" t="s">
+      <c r="G22" s="18"/>
+      <c r="H22" s="19" t="s">
         <v>102</v>
       </c>
       <c r="I22" t="s">
@@ -2164,17 +2149,17 @@
       <c r="B23" t="s">
         <v>139</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C23" s="17" t="s">
         <v>108</v>
       </c>
       <c r="E23" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="F23" s="18" t="s">
+      <c r="F23" s="17" t="s">
         <v>111</v>
       </c>
-      <c r="G23" s="24"/>
-      <c r="H23" s="20" t="s">
+      <c r="G23" s="18"/>
+      <c r="H23" s="19" t="s">
         <v>112</v>
       </c>
       <c r="I23" t="s">
@@ -2194,11 +2179,11 @@
       <c r="E24" t="s">
         <v>143</v>
       </c>
-      <c r="F24" s="18" t="s">
+      <c r="F24" s="17" t="s">
         <v>119</v>
       </c>
-      <c r="G24" s="24"/>
-      <c r="H24" s="20" t="s">
+      <c r="G24" s="18"/>
+      <c r="H24" s="19" t="s">
         <v>120</v>
       </c>
       <c r="I24" t="s">

</xml_diff>

<commit_message>
Ajout de points de test sur PCB
</commit_message>
<xml_diff>
--- a/Hardware/Matériel.xlsx
+++ b/Hardware/Matériel.xlsx
@@ -12,9 +12,6 @@
     <sheet name="XIAO ESP32" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
-  </extLst>
 </workbook>
 </file>
 
@@ -1421,7 +1418,7 @@
         <v>10</v>
       </c>
       <c r="F12" s="7">
-        <v>8.0000000000000002e-002</v>
+        <v>0.080000000000000002</v>
       </c>
       <c r="G12" s="2">
         <v>2</v>
@@ -1445,14 +1442,14 @@
         <v>10</v>
       </c>
       <c r="F13" s="7">
-        <v>8.0000000000000002e-002</v>
+        <v>0.080000000000000002</v>
       </c>
       <c r="G13" s="2">
         <v>1</v>
       </c>
       <c r="H13" s="8">
         <f t="shared" si="1"/>
-        <v>8.0000000000000002e-002</v>
+        <v>0.080000000000000002</v>
       </c>
     </row>
     <row r="14" ht="14.25">
@@ -1469,7 +1466,7 @@
         <v>10</v>
       </c>
       <c r="F14" s="7">
-        <v>8.0000000000000002e-002</v>
+        <v>0.080000000000000002</v>
       </c>
       <c r="G14" s="2">
         <v>2</v>

</xml_diff>